<commit_message>
Import 54 People from the People & Partners sheet into Community
- ImportPeopleSeeder reads assets/people.json (exported from the sheet),
  upserts Community records by name (sheet overwrites bio/photo when
  present, blank cells left untouched), and pulls each photo from its
  Google Drive link into the public disk
- community-single: preserve line breaks for plain-text bios (nl2br),
  leave existing HTML bios untouched

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/People and Partners.xlsx
+++ b/People and Partners.xlsx
@@ -11,102 +11,217 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="206">
   <si>
     <t>People</t>
   </si>
   <si>
-    <t>Job Descriptions</t>
+    <t>Short Bio</t>
+  </si>
+  <si>
+    <t>Full Bio</t>
+  </si>
+  <si>
+    <t>Pictures</t>
   </si>
   <si>
     <t>Partners</t>
   </si>
   <si>
+    <t>Photo</t>
+  </si>
+  <si>
+    <t>Bio</t>
+  </si>
+  <si>
     <t>Abdalla Ashraf</t>
   </si>
   <si>
     <t>Venture builder in international development, academia, consulting, and tech entrepreneurship</t>
   </si>
   <si>
+    <t>Abdalla Ashraf is a venture builder with a career spanning international development, academia, consulting, and tech entrepreneurship. He began by building university-based incubators (UBIs) globally, and later worked with UNDP, Strategy&amp;, and AUC on economic empowerment and sustainability. He holds a BSc in Mechanical Engineering and an MSc in Sustainable Development and Entrepreneurship from the American University in Cairo, and is currently pursuing an MBA with One League in partnership with Harvard and MIT, focusing on Data Science and AI.
+Abdalla is the founder of the Third Mission Venture Studio (TMVS), based on his master’s research on the evolution of entrepreneurship in universities. TMVS has spun off two startups: Zaher.AI, a platform for AI visibility and Generative Engine Optimization (GEO), and Blacksmith AI, an AI-driven text-to-CAD engineering copilot.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1KhaKYolBPnUG7D8mLw50NYsoEYTU-J6y</t>
+  </si>
+  <si>
     <t>Fairwork</t>
   </si>
   <si>
+    <t>https://drive.google.com/open?id=1wWtZ23o8lzSw8aiPmA9iuXrNnEEhwiH-</t>
+  </si>
+  <si>
+    <t>Fairwork is an international action-research initiative led by the Oxford Internet Institute and the WZB Berlin Social Science Centre, working to improve labour standards in the global digital economy. It assesses digital labour companies against five principles—Fair Pay, Fair Conditions, Fair Contracts, Fair Management, and Fair Representation—developed through an ILO-led process and endorsed by organisations representing over 27 million workers. Through a transparent and consistent scoring system, Fairwork generates robust, comparable evidence on working conditions while engaging directly with companies to support meaningful improvements.
+In doing so, Fairwork goes beyond measurement to act as a catalyst for systemic change. By combining rigorous research with market signalling, policy influence, and worker empowerment, it challenges business models that depend on insecure and unprotected work. Its work spans a wide range of sectors, from location-based services to cloudwork and AI-related labour, and has contributed to hundreds of documented improvements in working conditions across dozens of countries. Through its evaluations and ongoing engagement, Fairwork is helping to shape a digital economy that is more fair, accountable, and sustainable.</t>
+  </si>
+  <si>
     <t>Ahmad M. Awad</t>
   </si>
   <si>
     <t>Founder and Director, Phenix Center for Economic and Informatics Studies</t>
   </si>
   <si>
+    <t xml:space="preserve">Ahmad Awad is the founder and director of the Phenix Center for Economic and Informatics Studies in Amman, Jordan. He has dedicated most of his professional life to promoting and defending human rights, with a particular focus on socio-economic rights, labor rights, social justice, and inclusive development.
+He has supervised and contributed to numerous studies, research papers, policy briefs, and position papers addressing labor, social protection, economic reform, development, and the role of civil society in public policy and decision-making. At both the national and regional levels, he has worked to strengthen the participation of civil society organizations in shaping public debate and influencing policy processes on key economic and social issues.
+In recent years, he has placed growing emphasis on research related to the future of work, emerging forms of employment, and the transformations reshaping labor markets as a result of digitalization, automation, and technological change. His work explores non-standard work arrangements, platform-based labor, and the policy responses needed to address digital transformation in labor markets in ways that promote decent work, protect workers’ rights, and reduce social vulnerability.
+Ahmad Awad holds an MA in International Political Economy and is a member of a number of civil society networks and coalitions at the national, regional, and international levels. In 2018, he was honored by the Office of the United Nations High Commissioner for Human Rights as an exceptional human rights defender on the occasion of the 70th anniversary of the Universal Declaration of Human Rights.
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1V8blWEnhPttDiP9kPx0GOyGSdcLfOCHC</t>
+  </si>
+  <si>
     <t>Ahmed Al-Bassyouni</t>
   </si>
   <si>
     <t>Founder and CEO, Cloudilic</t>
   </si>
   <si>
+    <t>Ahmed Al-Bassyouni is the Founder and CEO of Cloudilic, an AI and automation company focused on building Agentic Process Automation platforms for enterprises and government organizations. He has a background in automation engineering and artificial intelligence, with experience delivering AI-powered solutions across sectors including finance, real estate, logistics, and public services. Ahmed leads the development of Dragify, a platform that enables organizations to deploy AI agents to automate complex workflows, integrate with enterprise systems, and improve operational efficiency. His work focuses on helping companies transition from manual processes to AI-driven operations.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1mL0XwOe7RiK1TkrkmzJHLmMp6cWZ67di</t>
+  </si>
+  <si>
     <t>Ahmed Fakhry</t>
   </si>
   <si>
     <t>Co-founder and CEO, Scale by AI</t>
   </si>
   <si>
+    <t>Co-founder and CEO at Scale by AI</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1uwX7iUdDw64mq_W_yOaDMs47sH0X7sLq</t>
+  </si>
+  <si>
     <t>Alessandro Giovanni Lamonica</t>
   </si>
   <si>
     <t>Adjunct Professor, Brussels School of Governance; Research Associate, School’s Centre for Security, Diplomacy and Strategy (CSDS); Director of the Public Policies Unit, Anna Lindh Foundation.</t>
   </si>
   <si>
+    <t>Alessandro G. Lamonica is an adjunct professor at the Brussels School of Governance, where he teaches MA-level courses on the theory and practice of public and cultural diplomacy. Bridging academia and policy, he serves as a Research Associate at the School’s Centre for Security, Diplomacy and Strategy (CSDS) and is currently the Director of the Public Policies Unit at the Anna Lindh Foundation.
+Alessandro holds a PhD in European Studies and International Relations from the Sant’Anna School of Advanced Studies. He has an extensive background in managing EU-funded research and has provided strategic consultancy to both governmental and non-governmental organisations on policy development.
+His previous leadership roles include serving as the co-founder and deputy director of the Jean Monnet Centre of Excellence in Cultural Relations and Diplomacy (CREDO) at the University of Siena and as a long-standing member of the Consortium Board of the European Commission’s Cultural Relations Platform.
+A foreign policy analyst by training, his research focuses on the EU’s external relations and the cultural determinants of agent behaviour in international relations.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Dy4SvIfqoW9B08iZ2sGSWebkiCd4kX_f</t>
+  </si>
+  <si>
     <t>Amr AboDraiaa</t>
   </si>
   <si>
     <t>CEO, Rology</t>
   </si>
   <si>
+    <t>Amr Abodraiaa, CEO of Rology, brings his experience as the Co-founder and CEO of TownSoft, along with his strategic roles at multiple entities. His leadership, coupled with his understanding of the market dynamics and operational excellence, is pivotal to guiding Rology towards its strategic vision.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1sOEQpwFgEIKjwIJu0vgH9KOZPsVP1NXm</t>
+  </si>
+  <si>
     <t>Amr Safwat</t>
   </si>
   <si>
     <t>Manager of the African Multilateral Affairs at the International Relations Central Department, Ministry of Communications and Information Technology (MCIT)</t>
   </si>
   <si>
+    <t xml:space="preserve">Mr. Amr Safwat is currently the Manager of the African Multilateral Affairs at the International Relations Central Department, Ministry of Communications and Information Technology (MCIT), Egypt.  He has more than 18 years of extensive experience in digital diplomacy, setting and implementing ICT for development initiatives with international development partners, and formulating policy recommendations on cooperation with regional and international stakeholders. 
+He has a long history of developing and managing partnerships with multi-stakeholders on the regional and international levels with a special focus on Africa. 
+Mr. Safwat leads MCIT’s continental outreach in Africa and is its official representative in the different African intergovernmental organizations. He spearheaded the development of the African Continental strategy on Artificial Intelligence through his chairmanship of the African Union Working Group. He is also leading the AI portfolio of the African Telecommunications Union (ATU) Working Group in preparations for the ITU Plenipotentiary Conference 2026. Moreover, he is the Chairman of the ATU’s Working Group mandated to develop the African common stance for ITU’s World Telecommunications Development Conference (WTDC) 2025.
+He holds a Master’s degree in Public Administration from the Lee Kuan Yew School of Public Policy, National University of Singapore and another Master’s degree in Euro – Mediterranean Studies from the Faculty of Economics and Political Science, Cairo University. 
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1oqTR-FTlYkKuky_h-ggcJTvCp5qiPuoI</t>
+  </si>
+  <si>
     <t>Asma Ben Hassen</t>
   </si>
   <si>
     <t>Sustainable Development Economist</t>
   </si>
   <si>
+    <t>Asma Ben Hassen  is an economist from Tunisia. She holds a postgraduate degree in economic sciences and is working on a doctoral on formalizing the informal economy She has ten years of experience in higher education, where she specialized in macro and microeconomic issues in labor economics, project management and evaluation, and business creation. Her work focused on creating sustainable economic development through the promotion of self employment and entrepreneurship. Asma has also worked as a consultant, diagnosing needs and developing training</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1UIqFzs9FlNzLum3tRJyfTXz-g50Nkv5O</t>
+  </si>
+  <si>
     <t>Ayah Bdeir</t>
   </si>
   <si>
     <t>CEO, Current AI</t>
   </si>
   <si>
+    <t>Ayah Bdeir is an entrepreneur, technology leader and public speaker who has dedicated her career to breaking down barriers between people and technology, first in hardware, then in education, and now in AI. 
+She is currently CEO of Current AI,  a $400M+ first-of-its-kind partnership bringing together governments, foundations, and the private sector, structured to prove that public interest AI can exist at scale.
+For the past 15 years, Bdeir’s work has centred around using technology to empower people to become changemakers, with a particular focus on underrepresented communities. Prior to joining Current AI, she led Mozilla’s AI strategy and worked across Mozilla (Mozilla Foundation, Mozilla Corporation, Mozilla Ventures, and Mozilla AI) to drive industry-defining collaborations towards open and trustworthy AI.
+Bdeir started her career in tech as founder and CEO of littleBits, the electronic building block that transformed STEAM education for millions of kids around the world. Under her leadership, littleBits generated over $150 million in lifetime revenue, won over 100 awards, including Toy of the Year, was used in 20,000 schools, and partnered with Disney, NASA and KORG. littleBits was acquired by Sphero in 2019.
+Bdeir was named one of BBC’s 100 Most Influential Women, was featured on 60 Minutes, and has appeared on the covers of The New York Times Magazine, WIRED and the Wall Street Journal. Her inventions are included in the permanent collection of The Museum of Modern Art (MoMA), and she holds over a dozen patents.
+Bdeir graduated from the MIT Media Lab and the American University of Beirut. She was a TED Fellow and serves on the board of the Fund for Public Schools, supporting NYC’s 1,800 public schools.
+At home in New York City, her 4 year old son makes her regret spending a decade advocating for kids to be mischievous.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=17xgBkOPqOw_rHwd0kC4g9kSIOZ-21x-q</t>
+  </si>
+  <si>
     <t xml:space="preserve">Doaa Salem Bashanfar </t>
   </si>
   <si>
     <t>Expert in continuing education, program development and partnerships</t>
   </si>
   <si>
+    <t xml:space="preserve">Dr. Doaa Salem has more than 20 years of experience in continuing education, program development and partnerships. She redefined the role of continuing education as a catalyst for inclusive economic transformation. Her pioneering partnership model uniquely integrates academia, government, the private sector, and grassroots organizations into a cohesive ecosystem that directly connects learning to opportunity. Unlike traditional approaches, her model is intentionally designed to reach underserved and marginalized communities, particularly women and youth, equipping them with practical, market-driven skills and clear pathways to employment, entrepreneurship, and career growth. Its strength lies in its scalability and adaptability, offering a replicable framework that can be applied across sectors and regions to drive sustainable socio-economic impact.
+International Recognition:
+This innovative approach has earned Dr. Salem international recognition, positioning her as a leading voice in the field of continuing education. Her model was selected for presentation at the UPCEA International Conference, placing Egypt on the global map of continuing education innovation and amplifying the contribution of Egyptian practitioners. Further affirming the global relevance of her work, Dr. Salem has been invited twice to Hong Kong to share her expertise with international audiences representing 36 nationalities. These engagements highlight the novelty, transferability, and global resonance of her partnership-driven model.
+Local Impact:
+ At its core, Dr. Salem’s model is grounded in inclusion and access, ensuring that women, youth, and individuals across diverse Egyptian governorates are not only reached, but meaningfully equipped with practical, market-relevant skills. Through deliberate and sustained collaboration with governmental entities, non-governmental organisations, and industry leaders, Dr. Salem has built an integrated ecosystem where education directly translates into opportunity. Her approach enables participants to transition seamlessly into employment, entrepreneurship, or career progression. It is especially impactful for individuals seeks advancement , offering them flexible, accessible, and context-responsive learning journeys. The impact extends well beyond individual beneficiaries: families experience improved livelihoods, and communities benefit from a more capable, resilient, and future-ready workforce.
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1i4ZU_7hlVXIyW4o7TuVN1te7-doajb-x</t>
+  </si>
+  <si>
     <t>Fola Adeleke</t>
   </si>
   <si>
     <t>Executive Director and Co-Founder, Global Center on AI Governance</t>
   </si>
   <si>
+    <t>Prof. Fola Adeleke is the Executive Director and co-founder of the Global Center on AI Governance. Fola leads our knowledge hub, the African observatory on Responsible AI. He holds a PhD in international investment law and human rights from the University of Witwatersrand and completed his post-doctoral research as a Fulbright Scholar at the Columbia Center on Sustainable Investment, Columbia University and the Human Rights Program, Harvard University.
+Fola is also an Associate Professor at Wits Law School South Africa, an Atlantic Senior Fellow on Social and Economic Equity at the London School of Economics and an Assistant Professor in Commercial Law at the Sobey Business School, St Mary's University, Canada. Fola currently serves as a Commissioner for the Lancet Commission on AI and HIV. Fola is an NRF rated researcher in South Africa and his research focuses on data protection, transparency, international investment law and corporate accountability</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1U-y-cFDT9QGucsquxyKuUa1C5q7KWbEv</t>
+  </si>
+  <si>
     <t>Gretchen King</t>
   </si>
   <si>
     <t>Associate Professor of Multimedia Journalism and Communication at Lebanese American University (LAU); Director of Pedagogy and Curriculum Design, LAU’s Institute of Media Research and Training</t>
   </si>
   <si>
+    <t xml:space="preserve">Associate Professor of Multimedia Journalism and Communication at Lebanese American University (LAU), Dr. Gretchen King also serves as the Director of Pedagogy and Curriculum Design at LAU’s Institute of Media Research and Training, where she is building a network of feminist AI enthusiasts. Since 1999, Dr. King has been working, teaching, and research at the intersection of politics and technology. She is the recent co-author of "The political economy of AI: a content analysis of ChatGPT outputs and anti-Palestinian media bias" published in Third World Quarterly. </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1bQPZAGGQle3Am2kDuqlKFKjG7UamDBs_</t>
+  </si>
+  <si>
     <t>Hala Gohar</t>
   </si>
   <si>
     <t>Marketing and Communications Director, Capgemini Egypt</t>
   </si>
   <si>
-    <t>Haya El Zayat</t>
-  </si>
-  <si>
-    <t>Senior Researcher, National Centre for Social Research (NatCen)</t>
+    <t>Hala Gohar is an accomplished Marketing and Communications leader with over 30 years of experience across major global technology companies. She currently serves as Marketing and Communications Director at Capgemini Egypt, where she built the function from the ground up and drives the brand’s visibility and strategic narrative. Her career spans senior roles at IBM, GB Auto, Alcatel‑Lucent, and Nortel, leading regional MARCOMS, CSR, corporate affairs, and executive profiling initiatives. She is recognized for her ability to shape brand reputation, build communication frameworks, and lead high‑impact campaigns that support business priorities. Hala holds a BA from the American University in Cairo and is passionate about fitness, wellness, and reading.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1KA3sFzIi0PkUWHpWS7Pjv9DcAg-sJDKS</t>
   </si>
   <si>
     <t>Isaac Rutenberg</t>
@@ -115,65 +230,126 @@
     <t>Advisor to the CEO at CIFOR-ICRAF; Associate Professor of ICT Policy and Innovation and Founder of Center for Intellectual Property and Information Technology Law (CIPIT), Strathmore University</t>
   </si>
   <si>
+    <t xml:space="preserve">Isaac Rutenberg is an Advisor to the CEO at CIFOR-ICRAF, an international science research institution based in Nairobi, Kenya. He has 20+ years of experience supporting innovation and innovators across sectors and geographies. He is an Associate Professor of ICT Policy and Innovation at Strathmore University in Nairobi, where he founded the Center for Intellectual Property and Information Technology Law (CIPIT) and served as its first Director from 2012-2022. At CIPIT, Prof. Rutenberg made contributions to global discussions around data governance, artificial intelligence, intellectual property, and contextualized innovation, particularly from the perspective of the Global South. Now at CIFOR-ICRAF, he is building a program supporting scientists and policymakers at the intersection of emerging technologies, agriculture, biodiversity, and climate change. </t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=10jZDgBZR1TGC0fO2_HirmjPwr2fIDc5L</t>
+  </si>
+  <si>
     <t>Karim Hamza</t>
   </si>
   <si>
     <t>AI Policy Strategist and Digital Governance Expert; Creator of the AIM-5 AI Leadership Maturity Framework</t>
   </si>
   <si>
+    <t>Dr. Karim is AI policy strategist and digital governance expert with over 25 years of experience advising governments, international institutions, and regulated industries on technology policy, economic competitiveness, and digital transformation.
+His work focuses on the intersection of artificial intelligence governance, economic policy, and institutional capacity, with particular attention to how emerging technologies reshape productivity, regulatory frameworks, and global competitiveness.
+He is the creator of the AIM-5 AI Leadership Maturity Framework, a governance model designed to help governments and institutions assess their readiness for responsible AI adoption across policy, infrastructure, talent, and innovation ecosystems.
+He had contributed to policy dialogue involving European institutions, governments, financial regulators, and international organizations, with a focus on AI governance, digital economy transformation, and institutional modernization.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=10R7FPDnyXH14GnShcTF8zkbQqamkK2ZI</t>
+  </si>
+  <si>
     <t>Khalid Choukri</t>
   </si>
   <si>
     <t>Founder and CEO, Evaluations and Language Resources Distribution Agency (ELDA); General Manager, Language Resources and Evaluation Conference (LREC)</t>
   </si>
   <si>
+    <t>Dr. Khalid Choukri is a Franco-Moroccan expert in language technologies and a key figure in the international NLP community. He has been the Secretary General of the European Language Resources Association (ELRA) and the Founder and CEO of the Evaluations and Language Resources Distribution Agency (ELDA) since 1995.
+He holds an engineering degree in Electrical Engineering (ENAC, Toulouse) and a Master’s and PhD in Computer Science and Signal Processing from Télécom Paris.
+With over 30 years of experience, his work focuses on spoken, written, and multimodal language technologies, particularly in multilingual and multicultural contexts, bridging academia and industry. He has been involved in nearly one hundred language resource collection projects worldwide, contributing to the creation, evaluation, and distribution of essential datasets for research and industry.
+Dr. Choukri has played a central role in the development of language technology infrastructures, standards, and international initiatives, and he served as Chair of ISO/IEC JTC 1/SC 35 (User Interfaces) for over 10 years. He has also been a key manager of numerous projects related to Artificial Intelligence, Natural Language Processing, and Arabic language technologies. In this context, he notably co-managed major projects such as NEMLAR and MEDAR, which contributed to advancing Arabic NLP and AI resources and technologies.
+He was among the founders of the Language Resources and Evaluation Conference (LREC) in 1998 and continues to act as its General Manager, contributing to its development as a leading international event in the field. He is currently involved in major European initiatives related to Large Language Models (LLMs), helping shape the future of multilingual AI in Europe and beyond.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1IjFyHf6n1xdpZt9HsW4ph13eE8ErwINI</t>
+  </si>
+  <si>
     <t>Lina Oueidat</t>
   </si>
   <si>
     <t>National Coordinator for Lebanon’s Cybersecurity Strategy, Counter-Terrorism Strategy, Cybersecurity Compendium, and Auditor for the Digital Transformation Strategy; Professor, Lebanese University (Faculties of Engineering and Law); Member, Women in Cybersecurity Middle East (WiCSME)</t>
   </si>
   <si>
+    <t xml:space="preserve">Dr. Lina Oueidat is an electronic and communication engineer, graduate of USJ (Lebanon) and ENSTA (France), with dual PhDs in Electronic Engineering and Biomedical Engineering from SUPELEC and Paris XI.-France She holds four European patents in engineering and medical fields, and a Master in Philosophy from the Lebanese University.
+Since 1995, she has served as senior advisor on ICT, Cybersecurity, and AI across multiple Lebanese ministries and institutions, including Public Health, Interior, Defense,Energy &amp; Water, Education, Defense, and the Presidency of the Council of Ministers, where she has been ICT advisor since 2012. She is National Coordinator for Lebanon’s Cybersecurity Strategy, Counter-Terrorism Strategy, Cybersecurity Compendium, and Auditor for the Digital Transformation Strategy.
+Member of the International Team drafting the Cloud Maturity Model (World Bank –UAE- Singapore)
+Internationally, Dr. Oueidat is a member of the International Cloud Computing Working Group and participates in the ITU-T Group on Security Standards validation (2025). She has advised organizations such as the EU, UNESCO, WHO, World Bank, UNODA, and KFAED, and currently serves as CT expert in an EU-funded project at the Presidency of the Council of Ministers.
+Dr. OUEIDAT is member of the Lebanese Committee of Professors that drafted the AI Ethics and Governance Guidelines- 2024.
+She is professor at the Lebanese University (Faculties of Engineering and Law), teaching AI, modern telecommunications, real-time embedded systems, modern physics, and decision-making. She has published extensively in cyber sciences, supervised doctoral research, and founded two consulting firms (ECS Consulting and EDITRA).
+PHD Co-advisor in AI , Cybersecurity and Quantum Computing PQC. 
+Dr. Oueidat is also a member of Women in Cybersecurity Middle East (WiCSME) and sings with the Antonine University Choir.
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=16Y9V8qG7qcOiM1VgE-gbOBhGmS5nx3P9</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maha Jouini </t>
   </si>
   <si>
     <t>Vice President, Agence Francophone et Africaine de l'Intelligence Artificielle (AFRIA); Digital Communication and Advocacy Lead, AUDA-NEPAD; Fellow Researcher, Francophone Africa; Fellow, Center for AI and Digital Policy (CAIDP)</t>
   </si>
   <si>
+    <t>Maha Jouini is a Global South AI thought leader, policy strategist, and digital transformation advocate with over a decade of experience working across Africa and the MENA region. Her work sits at the intersection of artificial intelligence, human rights, and inclusive development — anchored in an unwavering conviction that innovation must reflect dignity, justice, and the lived realities of African societies. As Vice President of the Agence Francophone et Africaine de l'Intelligence Artificielle (AFRIA) and digital communication and advocacy lead at AUDA-NEPAD, she shapes continental conversations on AI policy, responsible innovation, and Africa's digital sovereignty. At the Global Center on AI Governance, she serves as a Fellow Researcher advancing knowledge on Women and AI in Francophone Africa, and as a Fellow of the Center for AI and Digital Policy (CAIDP, 2022) and certified practitioner of Stanford Engineering's Ethics, Technology and Public Policy Program, she brings both institutional authority and field-level rigour to every platform she occupies.
+Her policy and advocacy work spans continents and communities. As a Researcher with the Global Index on Responsible AI, she conducted regional ethical risk assessments on Senegal's AI policies and engaged stakeholders to promote inclusive adoption. In Mauritania, she led mobile technology-driven digital literacy programs for uneducated women and girls in rural communities — closing education gaps where institutions had not reached. A finalist of the prestigious She Shapes AI Award and a published author on AI and economic development in both Arabic and English, she is especially recognized for championing culturally grounded AI governance — drawing on African philosophical frameworks such as Ubuntu and Hikma to make the case that technology must not only be intelligent, but wise.
+Her roots in human rights advocacy run deep. From championing migrant rights and GBV prevention at the Arab Institute for Human Rights in Tunisia, to serving as Regional Advocacy and Digital Communication Officer for the African Union's Campaign to End Child Marriage — advising the AU's Special Youth Envoy and shaping policy strategies that informed continental child protection frameworks — Maha has always understood technology as a tool for justice, not just growth. She began her career as a Blogger and Team Leader with Tunivisions during Tunisia's democratic transition in 2011, where she helped shape youth engagement at one of the most pivotal moments in the country's modern history.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1HIATj-1VRAbk9H9tTFk294_THzyadI5a</t>
+  </si>
+  <si>
     <t>Mahmoud Abdallah</t>
   </si>
   <si>
     <t>Advocacy and Programme Innovation Lead, Egyptian Food Bank (EFB)</t>
   </si>
   <si>
+    <t>(Side note: you can take the first paragraph in case the second makes it too long)
+Mahmoud Abdallah is the Advocacy and Programme Innovation Lead at the Egyptian Food Bank (EFB). He brings over 7 years of experience in research and policy analysis, project management, and collaboration with international organisations, think tanks, and academic institutions. His professional journey is defined by a commitment to evidence-based advocacy and a continuous pursuit of innovative frameworks that advance socio-economic development in Egypt and ensure long-term sustainability.
+At EFB, Mahmoud is part of the Policy Dialogue Initiative's (PDI) team, a platform dedicated to fostering evidence-based policy dialogues and stakeholder engagement. Through the PDI, he has facilitated engagements with regional and international stakeholders, including collaboration with the MENA Observatory on Responsible AI, positioning EFB as a credible voice in policy and advocacy circles across the region.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1WDMG-gh6A0UvglE3cbO2oPaph8vO11R_</t>
+  </si>
+  <si>
     <t>Marwa Soudi</t>
   </si>
   <si>
     <t>Consultant, MENA Observatory of Responsible AI at the American University of Cairo (AUC)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">Marwan Abdin | </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>https://linktr.ee/marwan.abdin</t>
-    </r>
+    <t>Marwa Samih Soudi is a distinguished researcher and innovator in the field of educational technology and artificial intelligence, with over 15 years of experience in the EdTech industry. Currently a PhD Candidate at Tallinn University, Marwa is pursuing her Ph.D. focusing on Responsible AI and the development of a trustworthy AI ecosystem for small and medium enterprises (SMEs). She is also a consultant at the MENA Observatory of Responsible AI at the American University of Cairo.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1jmRBvoLeqdpN99HmPY8-eJqowgGfGzE8</t>
+  </si>
+  <si>
+    <t>Marwan Abdin</t>
   </si>
   <si>
     <t>Founder and CEO, ACG (Abdin’s Consultancy Group); Founder, ACG Academies</t>
   </si>
   <si>
+    <t>Marwan Abdin is the Founder and CEO of ACG (Abdin’s Consultancy Group), an Enterprise AI and management consulting firm with a strong footprint across MENA. He advises governments, multinationals, and startups on AI strategy, digital governance, and large-scale transformation. Marwan is actively engaged in global AI policy dialogues, including participation in United Nations discussions on the Global Dialogue on AI Governance, and has led and supported EU-backed AI hackathons, driving innovation across sectors such as water, agribusiness, and emerging technologies in the region. Marwan has support hackathons in evaluating the Technology Readiness levels and Open Innovations profiles in startups in fields such as agri-Tech, Water-Tech, Solar-tech, Med-Tech, Ed-Tech and Space-Tech. 
+He is also the Founder of ACG Academies, a dynamic portfolio of specialized academies including The AI Academy, Leadership X Academy, Future of Work Academy, The Retail Academy, and partner in TalentRise Academy, designed to empower individuals and organizations with future-ready skills, leadership capabilities, and AI-driven transformation.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1M8uWjcfcBiv6hWaoGh9_KKj-ABchfvpE</t>
+  </si>
+  <si>
     <t>Meriem Mehri</t>
   </si>
   <si>
     <t>Researcher in AI governance and human-AI interaction (HAII)</t>
+  </si>
+  <si>
+    <t>Researcher in AI governance and human-AI interaction (HAII), focused on designing responsible and human-centered systems. My work explores how technology can better support coordination, ethics, and collective well-being, with the intention of contributing to meaningful and lasting impact.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1UTCXvWTSD-2jtpQdKJQbeQwIaTlZR8p6</t>
   </si>
   <si>
     <t>Mia Negru</t>
@@ -183,6 +359,14 @@
 </t>
   </si>
   <si>
+    <t>Mia Negru is the Executive Director of Life With Artificials, an initiative focused on advancing the responsible integration of artificial intelligence and emerging technologies into society. Her work sits at the intersection of technology, policy, and public engagement, with a particular emphasis on trust, ethics, and human-centered innovation.
+With a background in political affairs and a strong interest in exponential technologies, Mia builds bridges between researchers, innovators, and policymakers to foster more inclusive and informed dialogue around AI. She is also the driving force behind the concept of SDG 18: Life With Artificials, advocating for a global framework to guide the societal impact of advanced technologies.
+Through her work, Mia contributes to shaping conversations on responsible AI by promoting accessibility, critical thinking, and cross-sector collaboration.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1k03OSloz55VAzMDvQrePdmQNOJj2rh50</t>
+  </si>
+  <si>
     <t>mohab said</t>
   </si>
   <si>
@@ -190,113 +374,252 @@
 </t>
   </si>
   <si>
+    <t>Mohab Said is an economist and business consultant, and the co-founder of SynQanun AI, an AI-powered legal technology platform designed to enhance access to legal knowledge and streamline legal research. His work focuses on leveraging artificial intelligence to bridge gaps between complex legal systems and practical, user-friendly applications for professionals and institutions.
+Through SynQanun AI, Mohab is developing data-driven solutions that enable faster, more accurate interpretation of legal documents and regulations, contributing to the modernization of legal services in Egypt and the wider region. His approach combines economic analysis with technology to improve efficiency, transparency, and decision-making within legal and regulatory environments.
+In addition to his work in legal tech, Mohab has extensive experience in economic development, employability, and policy-oriented research through his role at Manifesto Consultancy, where he has contributed to projects supporting entrepreneurship, SMEs, and inclusive growth across the MENA region.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1_QU6JxfPc2t_baz5TKeT2uwUAVlGkhuw</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mohamed Abdelgawad </t>
   </si>
   <si>
     <t>Co-Founding Partner and Head of the Corporate, Commercial and Regulatory department, ADSERO – Ragy Soliman &amp; Partners</t>
   </si>
   <si>
+    <t>Mohamed is a Co-Founding Partner at ADSERO – Ragy Soliman &amp; Partners. He heads the firm’s Corporate, Commercial and Regulatory department. Although Mohamed has diversified experience in multiple legal disciplines, including corporate M&amp;A, projects and finance, dispute resolution, and general corporate and commercial legal services, he is now focused on leading the firm’s non-transactional corporate and commercial matters.
+Mohamed has broad expertise in general corporate and commercial matters, including contracts law, regulatory and compliance, services agreements, licensing and IP, franchising, employment and anti-bribery.
+Mohamed has developed a market lead in the TMT and life sciences sectors with several landmark transactions and a solid base of strategic clients. In addition, Mohamed regularly advises most prominent technology and telecommunications companies on various legal matters, including cyber security data protection, fintech and electronic signature.
+Mohamed is identified as a market expert in the life sciences sector. He has advised on the Egyptian aspects of most global transactions in the pharmaceutical industry in the past decade.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1nFFOzyC4ALUULz7EXzoxLKNsGuWBBwDX</t>
+  </si>
+  <si>
     <t>Mohamed Nekhely</t>
   </si>
   <si>
     <t>Digital Innovation Director</t>
   </si>
   <si>
+    <t>Mohamed El Nekhely is a Digital Innovation Director with 20+ years of experience leading AI-driven digital transformation and building transparent, data-driven solutions that enhance impact in the humanitarian sector.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1KpAwfYpLP5LSJkJD2F6gxyh5LvwbY57n</t>
+  </si>
+  <si>
     <t>Mohamed Zahran</t>
   </si>
   <si>
     <t>Computer Science Department Faculty Member, NYU; Senior Member, IEEE; Senior Member, ACM</t>
   </si>
   <si>
-    <t xml:space="preserve">mona ezat </t>
+    <t>Mohamed Zahran is currently a faculty member with the Computer Science Department at NYU. He received his Ph.D. in Electrical and Computer Engineering from University of Maryland at College Park in 2003. His research interest spans several aspects of computer hardware design, hardware/software interaction, and high-performance computing. Zahran is a senior member of IEEE, senior member of ACM,  and  Sigma Xi scientific honor society.
+He is also a non-fiction writer with a weekly column on Al-Shorouk magazine where he writes about science, history of science, scientific and academic life.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1S0FT0CCt7CQSiSQBtpfSdPZHrT5lLyMy</t>
+  </si>
+  <si>
+    <t>Mona Ezat</t>
   </si>
   <si>
     <t xml:space="preserve">Founder, Al-Noon Foundation for Family Care; Member of the NGO Committee and Coordinator of the Economic Empowerment and Financial Inclusion Working Group, National Council for Women; Member, Arab States Civil Society Oganizations and Feminist Network; Member, Global Network for Economic, Social and Cultural Rights
 </t>
   </si>
   <si>
+    <t xml:space="preserve">-Founder/Al-Noon Foundation for Family Care
+-Master of Business Administration, marketing specialty,  Sadat Academy for  Administrative Sciences,2020
+-Member of the NGO Committee of the National Council for Women/ Coordinator of the Economic Empowerment and Financial Inclusion Working Group ,from 2016 to date
+- member the Arab states   Civil Society organizations and  Feminist Network 
+-  Member of the Global Network for Economic, Social and Cultural Rights
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1VWS0e_Qmj1PCJKxwnlw1WebqXpWBmWQs</t>
+  </si>
+  <si>
     <t>Mostafa ElAwamy</t>
   </si>
   <si>
     <t>Lead, Digital Products Design and Engineering Unit</t>
   </si>
   <si>
+    <t>https://drive.google.com/open?id=1jxk9qx4eEZsBkL5ptFaCYTJRt4saWUFU</t>
+  </si>
+  <si>
     <t>Nada Alwadi</t>
   </si>
   <si>
     <t>Ph.D. student at Virginia Tech, specializing in Planning, Governance, and Globalization</t>
   </si>
   <si>
+    <t>Nada Alwadi is a Ph.D. student at Virginia Tech, specializing in Planning, Governance, and Globalization, with a research focus on the Arab Gulf States. 
+Her research delves into the future of governance in the digital era, specifically exploring how emerging technologies are reshaping power dynamics, policymaking, and societal development.
+Previously, Nada served as a Team Leader at the Center for Artificial Intelligence and Digital Policy (CAIDP) in Washington, D.C., where she earned an Advanced Certificate in AI Policy. During her time at the Center, she was integral to updating the Artificial Intelligence and Democratic Values Index for 2025 and 2026.
+In addition to her academic and professional accomplishments, Nada is an award-winning journalist and storyteller, passionate about the intersection of technology, governance, and human rights. Her work aims to foster global conversations around digital rights and the ethical implications of emerging technologies on governance and policy .</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1raKOkT-pz1ie0DTuRBPN3CPiHyOdg4Dt</t>
+  </si>
+  <si>
     <t>Nagwa ElSayed</t>
   </si>
   <si>
     <t>Head of the Scientific Research and Innovation Sector, Misrelkheir Foundation</t>
   </si>
   <si>
+    <t xml:space="preserve">Nagwa A. ElSayed has been working in the field of scientific research project funding since 2008. Nagwa is currently working as the head of the Scientific Research and Innovation Sector at Misrelkheir Foundation. She is responsible for many programs to fund world-class scientific research projects with high societal impact and promote the culture of scientific research and innovation and support innovators and technology startups solving social challenges. Previously, she worked in the Science and Technology Development Fund (STDF) in the Planning and Monitoring Department from 2008 to 2011, where she was responsible for reporting about STDF’s status to the management and monitoring STDF achievements in alignment with the plan. 
+From 2002 to 2008, she worked in the Science and Technology Center in the Academy of Scientific Research and Technology in the information technology field. From 1990 till 2002 she worked in several USAID projects in the field of information technology with the Academy of Scientific Research and Technology, Egyptian Electricity Authority, and the Ministry of Industry and Foreign Trade. 
+Nagwa holds a Doctor of Business Administration (DBA) in Strategic Management from the American International Theism University, a Master's in Business Administration (MBA) from the International Business Administration of Switzerland (IBAS) and a Diploma in Management of Technology from Nile University. She is a Microsoft Certified System Engineer and has a B.Sc. in Computer Science from the American University in Cairo. She took several courses in Project Management Professional (PMP), Millennium Manager, and strategic planning for NGOs.
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1-HKTVe2ZV7GJNtOzXlxl6lspsVsV_-59</t>
+  </si>
+  <si>
     <t>Nezar Sami</t>
   </si>
   <si>
     <t>Skills Development Analyst at the Knowledge Project, United Nations Development Programme (UNDP)</t>
   </si>
   <si>
+    <t xml:space="preserve">Nezar Sami is a Skills Development Analyst at the Knowledge Project of the United Nations Development Programme (UNDP).
+A learning, innovation, and technology management expert, he brings over 30 years of experience delivering national and regional development programmes, digital transformation projects, innovation and entrepreneurship initiatives across public and international institutions. 
+Sami contributes to the design and implementation of the Future Skill Academy, providing technical and operational leadership across youth skilling, research, and innovation in learning. His work includes contributing to research agendas, skills gap mapping, and evidence-based policy products in close coordination with UNDP country offices. 
+Additionally, he leads strategic stakeholder engagement across government, the private sector, and academia to align research with regional innovation agendas.
+Previously, he held senior leadership positions at UNDP Egypt, Nile University, and the Egyptian Banking Institute; he also founded the NilePreneurs initiative.
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1QIgclsC4v89pN1iWtPaheyUKX_zcT0BN</t>
+  </si>
+  <si>
     <t xml:space="preserve">Noha Abdel-Hamid </t>
   </si>
   <si>
     <t>Technical Facilitator, UNDP Egypt Country Office; Financial Inclusion Expert, COSPE ONLUS</t>
   </si>
   <si>
+    <t>Noha Abdel HamidNoha Abdel Hamid is an accomplished international business and purpose leader with extensive experience in driving social impact through innovative solutions. With a strong focus on women's entrepreneurship, economic empowerment, and financial inclusion, she has successfully founded two nonprofit organizations dedicated to supporting women.Currently, Noha serves as a Technical Facilitator at the UNDP Egypt Country Office, where she leads discussions on child marriage and its implications for society. Additionally, she is a Financial Inclusion Expert with COSPE ONLUS, promoting equitable access to financial resources for women across the MENA region through the InclusiveNissa program.Her background includes significant roles in partnerships and advocacy with organizations such as Plan International and CARE International, where she managed advocacy initiatives and built strategic partnerships with the private sector. Noha's expertise extends to board management, governance, proposal writing, and public speaking, making her a sought-after mentor and coach for aspiring entrepreneurs and NGOs.Noha holds a Master’s degree in Public Policy &amp; Administration from the American University in Cairo and is actively pursuing accreditation as a Professional Coach. Her commitment to empowering women and promoting financial literacy has made her a prominent figure in the field, contributing to various training programs and workshops across the region.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1ixks8N4c7gq_p5Fe5-4peViiYikh44tA</t>
+  </si>
+  <si>
     <t>Nour Naim</t>
   </si>
   <si>
     <t>Founder, AI Minds Academy</t>
   </si>
   <si>
+    <t>Dr. Nour Naim is an AI Business Manager and specialist in AI Governance, Risk, and Compliance (GRC), holding a Ph.D. in AI Management with a focus on the socio-technical and ethical dimensions of autonomous systems. She leads AI strategy and governance initiatives at Dataliva, collaborates independently with Columbia University on AI ethics research, and teaches AI Ethics at Istanbul Yeni Yüzyıl University. She is also the Founder of AI Minds Academy, where she works to advance responsible AI ecosystems in the SWANA region and advocates for ethical governance and inclusive global AI representation.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1yc3E0dJ50PFXE4HqQ0HCLN68_N9ihSyF</t>
+  </si>
+  <si>
     <t>Osama Attia</t>
   </si>
   <si>
     <t>Co-Founder &amp; CEO of DATAGENX</t>
   </si>
   <si>
+    <t>I'm Osama Attia is the Co-Founder &amp; CEO of DATAGENX, specializing in data management solutions and tools. With over 10 years of experience in business development and operations</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1cyOlaA_eGOeR2_dP6zfmWpVNz1ZvV-i8</t>
+  </si>
+  <si>
     <t>Paola Ricaurte Quijano</t>
   </si>
   <si>
     <t>Full Profeesor, Tecnológico de Monterrey; Faculty Associate at the Berkman Klein Center for Internet &amp; Society, Harvard University; Co-founder, Tierra Común</t>
   </si>
   <si>
+    <t>Paola Ricaurte is a full professor at Tecnológico de Monterrey and a faculty associate at the Berkman Klein Center for Internet &amp; Society at Harvard University. She is the co-founder of Tierra Común, an academic and activist network committed to decolonizing data, and leads the Latin American and Caribbean Feminist AI Network. Paola serves on several international expert committees, including the Global Partnership on AI (GPAI), UNESCO’s AI Ethics Experts Without Borders (AIEB), and the Women for Ethical AI (W4EAI) platform. She was included in the 2025 TIME100 AI list of the most influential people in artificial intelligence.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1RPYExP0d_Bks8zx9KMlFOvaYEBYyvIy5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sahar Albazar </t>
   </si>
   <si>
     <t>Egyptian Member of Parliament; Deputy Chair of Foreign Affairs Committee, Egyptian Parliament; Vice President, Africa AI Forum; Volunteer Advisor to the Cabinet of Pakistan on AI policy</t>
   </si>
   <si>
+    <t>Sahar Albazar is an Egyptian Member of Parliament &amp; the Deputy Chair of Foreign Affairs Committee at the Parliament. Albazar is a global leader in artificial intelligence policy, digital governance, and emerging technologies. She currently serves as the Egypt Country Director at the Global AI Council, where she leads national engagement on AI strategy, partnerships, and policy alignment with global standards.
+At the continental level, she is the Vice President of the Africa AI Forum, contributing to shaping Africa’s collective voice on AI governance, innovation ecosystems, and inclusive digital transformation.
+Internationally, Sahar serves as a Volunteer Advisor to the Cabinet of Pakistan on AI policy, supporting the development of forward-looking regulatory frameworks and national AI strategies. She has also worked closely with the Egyptian government on AI policy, contributing to national efforts to integrate artificial intelligence into economic development, public services, and governance systems.
+Her work focuses on bridging policy and implementation—ensuring that AI is deployed responsibly to drive economic growth, improve public sector efficiency, and promote social inclusion. She brings a unique combination of legislative experience, international policy engagement, and cross-regional collaboration across Africa, the Middle East, and Asia.
+Sahar is also a World Economic Forum Young Global Leader, Yale World Fellow, and Harvard Kennedy School graduate, with a strong track record in shaping global conversations on technology, governance, and development.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1ayyW9Um1bLpQm9XDRAtQHGyQtNRsDbTE</t>
+  </si>
+  <si>
     <t>Salwa Tohme Tawk</t>
   </si>
   <si>
     <t>Professor of Agriculture Economics Farming Systems, Lebanese University</t>
   </si>
   <si>
+    <t>Salwa Tohmé Tawk studied at the American University of Beirut and completed a M.Sc. in Plant Production and Protection; she holds a “Diplôme en Etudes Approfondies” and PhD in Farming Systems and Sustainable Development from the "Institut National de Recherche Agronomique Paris-Grignon France". She is an agriculture engineer and a professor in agriculture economics farming systems. Her research and involvement in development projects focus on communication platform development, Regional Diagnosis, Post-harvest Losses, Business Planning, Needs &amp; Value chain assessment. She carried out, as a researcher, studies to understand and improve Food security in rural and urban settings, but also to promote a resilient and sustainable food system in Lebanon, Jordan and Yemen; she also works on program development for capacity building and is a capacity building expert on business management for farmers and cooperatives.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=15gU04prS0mwVTbOSHL7UsFHNdK98d43q</t>
+  </si>
+  <si>
     <t>Sameh Elbagoury</t>
   </si>
   <si>
     <t>Head for Saudi Arabia &amp; the Gulf, Sandoz</t>
   </si>
   <si>
+    <t xml:space="preserve">
+Sameh El‑Bagoury is a senior pharmaceutical leader and Head for Saudi Arabia &amp; the Gulf at Sandoz. With +25 Years of experience spanning General Management, commercial excellence, digital transformation, and emerging markets, he has led businesses across MENA, APAC, and Europe. He is passionate about leadership, healthcare access, and the thoughtful use of AI in decision‑making</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1mpmiDh28uB7lyBG2C1SVi8wwSOCDcQph</t>
+  </si>
+  <si>
     <t>Shady Elbassuoni</t>
   </si>
   <si>
     <t>Associate Professor of Computer Science and Chair of the Department, American University of Beirut (AUB); Academic Director, AUB’s Online Graduate Professional Diploma in AI and Data Science</t>
   </si>
   <si>
+    <t>Shady Elbassuoni is an Associate Professor of Computer Science at the American University of Beirut (AUB), where he also serves as Chair of the Department. He is the Academic Director of AUB’s Online Graduate Professional Diploma in AI and Data Science. He received his PhD from the Max Planck Institute for Informatics in Germany and completed a postdoctoral fellowship at Qatar Computing Research Institute.
+His research lies at the intersection of artificial intelligence and societal impact, with a focus on natural language processing (particularly Arabic NLP), AI for health, and AI ethics. His recent work explores the use of machine learning and computer vision to study food environments and public health, as well as issues of fairness, accountability, and transparency in AI systems.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1zuRjg1hu1067nezQTW5Q_EZAGZDl783d</t>
+  </si>
+  <si>
     <t>Shady Hamadeh</t>
   </si>
   <si>
     <t>Professor at the Faculty of Agricultural and Food Sciences, American University of Beirut (AUB); Founder and Director, Environment and Sustainable Development Unit (ESDU)</t>
   </si>
   <si>
+    <t>Prof. Hamadeh is a professor at the Faculty of Agricultural and Food Sciences at the American University of Beirut and serves as the founder and Director of the Environment and Sustainable Development Unit (ESDU). He is a leading expert in sustainable agriculture and animal science, with extensive experience in research, teaching, and development projects across Lebanon and the region. His work focuses on improving the resilience of food systems and rural livelihoods. Prof. Hamadeh also serves on several national advisory boards, contributing to policy dialogue and strategic direction on sustainable food systems and environmental management.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=145r5PaE_SMBNad4keeB3v2k6eAA5Uw-g</t>
+  </si>
+  <si>
     <t>Shahdan Arram</t>
   </si>
   <si>
     <t>Secretary General, Vodafone Egypt Foundation</t>
+  </si>
+  <si>
+    <t>Shahdan leads Vodafone Egypt Foundation’s ambitious mission to empower communities and create social impact through technology and innovation, working to improve youth access to knowledge and skills through formal and non-formal learning opportunities, as well as leveraging technology in the development of the health sector and in emergency response. With a deep-rooted passion for social impact, Shahdan has spearheaded numerous initiatives that bridge the digital divide and create opportunities for vulnerable populations in Egypt. Under her leadership, the Vodafone Egypt Foundation has grown its footprint significantly, developing strategic partnerships with government agencies, NGOs, private sector players, and local foundations to deliver impactful and scalable. Throughout her tenure, Shahdan has championed programmes and initiatives that improve digital literacy, AI, as well as increase access to quality education, and promote the culture of entrepreneurship. With over 20 years of professional experience in the development sphere, working for UN agencies, bilateral-donors and civil society organizations, she has driven strategic change across programmes in the fields of youth empowerment, education, Edtech, gender equality and civic engagement.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/171Uw3mPpYbtmW11vy5g5NkOqfdF4_hUC/view?usp=drive_link</t>
   </si>
   <si>
     <t xml:space="preserve">Sherif Ali Shalan </t>
@@ -318,10 +641,29 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">Sherif Ali Shalan is a seasoned entrepreneur, angel investor, and board member with a passion for the AI and data economy. As the Founder and CEO of PIANAT.ai, he leads a mission to transform how organizations in emerging markets approach governance, risk, and compliance through the power of artificial intelligence and data science.
+With over 20 years of executive leadership experience spanning the MENA region and the United States, Sherif has built a career defined by innovation, impact, and an unwavering commitment to enabling institutions and economies to make better, faster, and more informed decisions. His expertise encompasses artificial intelligence, data science, government relations, business strategy, and digital transformation.
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1XazrtYQRnI3eVe2nFfSIC0HivTdWvwbL</t>
+  </si>
+  <si>
     <t>Stephanie Boustany</t>
   </si>
   <si>
     <t>Project, Research and Communications Specialist, UNDP Regional Bureau for Arab States</t>
+  </si>
+  <si>
+    <t>Stéphanie Boustany – Project, Research and Communications Specialist, UNDP Regional Bureau for Arab States
+Stéphanie Boustany is a development professional with over 12 years of experience at UNDP’s Regional Bureau for Arab States, focusing on knowledge, skills development, and sustainable development.
+In her current role, she contributes to the design, implementation, and strategic positioning of the Knowledge Project, a flagship partnership between UNDP and the Mohammed bin Rashid Al Maktoum Knowledge Foundation. Her work includes leading initiatives such as the Global Knowledge Index, and coordinating research, data analysis, and communications efforts that inform policy dialogue and decision-making at regional and global levels.
+Stéphanie has extensive experience in development research, index design, and the production of evidence-based knowledge products. She works closely with policymakers, international organizations, academia, and private-sector partners to ensure that data and insights are translated into practical and policy-relevant outputs.
+Her areas of expertise include data analysis, development research, composite indices, strategic communications, and knowledge-for-development programming.
+Stéphanie holds an MSc in Sustainable Development from SOAS University of London and a BA in Economics from Notre Dame University, Lebanon.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1BxOaRbXOm1ibU7zLsr08IPX8sAMKrNTe</t>
   </si>
   <si>
     <t>Usama Najeeb</t>
@@ -331,29 +673,72 @@
 </t>
   </si>
   <si>
+    <t xml:space="preserve">Usama Najeeb is a political and economic specialist with extensive experience analyzing governance, technology, and economic developments in the Middle East and North Africa. He has served at the U.S. Consulate in Dubai since 2018 and previously worked as a Political Specialist at the U.S. Embassy in Cairo from 2007 to 2018, focusing on political and economic reforms, regulatory frameworks, and regional cooperation. Usama is also a Chartered Linguist and Translator (CIOL) and a member of the American Translators Association, with a strong passion for translation and cross-cultural communication. He holds a Master of Arts in Journalism and Mass Communication from the American University in Cairo and a Diploma in International Water Law from the University of Geneva. A recipient of the Kamal Adham Fellowship for Television and Digital Journalism, he has lived between Egypt and the UAE since 1980.
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1Q8VmZXsbfI_D_bkdX0uHLpxanH7Ghm_9</t>
+  </si>
+  <si>
     <t>Yousif Hassan</t>
   </si>
   <si>
     <t>Assistant Professor of Public Policy at the Ford School of Public Policy, University of Michigan; Assistant Professor of Information in the School of Information, University of Michigan</t>
   </si>
   <si>
+    <t xml:space="preserve">Yousif Hassan is assistant professor of Public Policy in the Ford School of Public Policy and assistant professor of Information in the School of Information at the University of Michigan. His research focuses on the social, economic, and political implications of emerging technologies including artificial intelligence, machine learning, and natural language processing, with a particular emphasis on technoscientific innovation, development, and the digital economy. Hassan’s interest is at the intersection of social justice and technology policy. His most recent work investigates the development of AI and its innovation ecosystem across multiple African countries focusing on AI, data governance, and the data economy.  
+Hassan received his B.Sc. in Electrical and Electronic Engineering from University of Khartoum and Master of Engineering from McMaster University. He received his MA and PhD in Science and Technology Studies from York University.
+Hassan is a former Illinois distinguished fellow at the School of Information Sciences, University of Illinois Urbana-Champaign. He was a research fellow at the Kennedy School of Government, Harvard University. 
+</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1q0y90agb-USgnMVzbx8m7TTiXaI6uTS2</t>
+  </si>
+  <si>
     <t>Yusra Ahmad</t>
   </si>
   <si>
     <t>Founding Partner, Acuity Data</t>
   </si>
   <si>
+    <t>Yusra Ahmad is Founding Partner of Acuity Data, where she delivers  advisory services and training on AI governance and ethics to organisations across government and enterprise sectors. Former Chair of the RED Foundation's Data Ethics Committee, she has 18+ years of experience in digital transformation, having advised government entities including the UK Cabinet Office and NEOM, as well as Fortune 500 corporations including CBRE and HSBC. Yusra is a published author on data ethics and AI governance, with peer-reviewed work including "We are the makers of manners: A grounded approach to data ethics for the built environment" and the Data Ethics Playbook. She has contributed to AI policy research including work with the Global Index for Responsible AI.</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/open?id=1uXgIk5jREgiux6fnn_v36abuFOuPY1rK</t>
+  </si>
+  <si>
     <t>Hana Gad</t>
   </si>
   <si>
-    <t>Research Assitant</t>
+    <t>Research Assistant, Access to Knowledge for Development Center (A2K4D)</t>
+  </si>
+  <si>
+    <t>Rinad Ghaith</t>
+  </si>
+  <si>
+    <t>Research and Engagement Specialist, Access to Knowledge for Development Center (A2K4D)</t>
+  </si>
+  <si>
+    <t>Aliaa Hashim</t>
+  </si>
+  <si>
+    <t>Marize Gouda</t>
+  </si>
+  <si>
+    <t>Jessica Lamie</t>
+  </si>
+  <si>
+    <t>Basma Balabel</t>
+  </si>
+  <si>
+    <t>Nouran Hassan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -371,14 +756,32 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
     </font>
     <font>
       <u/>
@@ -401,24 +804,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF8F9FA"/>
+        <bgColor rgb="FFF8F9FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFB7B7B7"/>
         <bgColor rgb="FFB7B7B7"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8F9FA"/>
-        <bgColor rgb="FFF8F9FA"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FFF8F9FA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFF8F9FA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFF8F9FA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFF8F9FA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -432,32 +849,62 @@
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -510,10 +957,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A2:B50" displayName="Table_1" name="Table_1" id="1">
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A2:D56" displayName="Table_1" name="Table_1" id="1">
+  <tableColumns count="4">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
+    <tableColumn name="Column3" id="3"/>
+    <tableColumn name="Column4" id="4"/>
   </tableColumns>
   <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
@@ -720,7 +1169,10 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="24.88"/>
+    <col customWidth="1" min="1" max="1" width="34.63"/>
+    <col customWidth="1" min="2" max="3" width="55.0"/>
+    <col customWidth="1" min="4" max="4" width="83.88"/>
+    <col customWidth="1" min="8" max="8" width="24.63"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -730,14 +1182,22 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2"/>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
@@ -752,414 +1212,793 @@
       <c r="T1" s="2"/>
       <c r="U1" s="2"/>
       <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
-      <c r="Z1" s="2"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>7</v>
+      <c r="A3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>9</v>
+      <c r="A4" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>13</v>
+      <c r="A6" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>15</v>
+        <v>31</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>17</v>
+      <c r="A8" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>19</v>
+        <v>39</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>21</v>
+      <c r="A10" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>23</v>
+        <v>47</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>25</v>
+        <v>51</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>27</v>
+      <c r="A13" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>29</v>
+        <v>59</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>31</v>
+      <c r="A15" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>33</v>
+      <c r="A16" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>35</v>
+      <c r="A17" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>37</v>
+      <c r="A18" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>39</v>
+      <c r="A19" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>41</v>
+      <c r="A20" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>43</v>
+      <c r="A21" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>45</v>
+      <c r="A22" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>47</v>
+      <c r="A23" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>49</v>
+      <c r="A24" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>51</v>
+      <c r="A25" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>53</v>
+      <c r="A26" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>55</v>
+      <c r="A27" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>57</v>
+      <c r="A28" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>59</v>
+      <c r="A29" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>61</v>
+      <c r="A30" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B30" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="C30" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>63</v>
+      <c r="A31" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>65</v>
+      <c r="A32" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>67</v>
+      <c r="A33" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>69</v>
+      <c r="A34" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>71</v>
+      <c r="A35" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>73</v>
+      <c r="A36" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>75</v>
+      <c r="A37" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>77</v>
+      <c r="A38" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>79</v>
+      <c r="A39" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="D39" s="18" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="s">
-        <v>80</v>
+        <v>161</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>81</v>
+        <v>162</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>83</v>
+      <c r="A41" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="C41" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="D41" s="17" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B42" s="9" t="s">
-        <v>85</v>
+      <c r="A42" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="D42" s="18" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>87</v>
+      <c r="A43" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="C43" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="D43" s="17" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>89</v>
+      <c r="A44" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B44" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="D44" s="18" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>91</v>
+      <c r="A45" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="D45" s="17" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>93</v>
+      <c r="A46" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D46" s="18" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>95</v>
+      <c r="A47" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="C47" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="D47" s="17" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B48" s="9" t="s">
-        <v>97</v>
+      <c r="A48" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="D48" s="18" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="s">
-        <v>98</v>
+      <c r="A49" s="20" t="s">
+        <v>197</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>99</v>
-      </c>
+        <v>198</v>
+      </c>
+      <c r="C49" s="4"/>
+      <c r="D49" s="23"/>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="s">
-        <v>100</v>
+      <c r="A50" s="20" t="s">
+        <v>199</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>101</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="C50" s="4"/>
+      <c r="D50" s="23"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B51" s="23"/>
+      <c r="C51" s="23"/>
+      <c r="D51" s="23"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B52" s="23"/>
+      <c r="C52" s="23"/>
+      <c r="D52" s="23"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B54" s="23"/>
+      <c r="C54" s="23"/>
+      <c r="D54" s="23"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B55" s="23"/>
+      <c r="C55" s="23"/>
+      <c r="D55" s="23"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="23"/>
+      <c r="C56" s="23"/>
+      <c r="D56" s="23"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A23"/>
-    <hyperlink r:id="rId2" ref="B45"/>
+    <hyperlink r:id="rId1" ref="D2"/>
+    <hyperlink r:id="rId2" ref="D3"/>
+    <hyperlink r:id="rId3" ref="D4"/>
+    <hyperlink r:id="rId4" ref="D5"/>
+    <hyperlink r:id="rId5" ref="D6"/>
+    <hyperlink r:id="rId6" ref="D7"/>
+    <hyperlink r:id="rId7" ref="D8"/>
+    <hyperlink r:id="rId8" ref="D9"/>
+    <hyperlink r:id="rId9" ref="D10"/>
+    <hyperlink r:id="rId10" ref="D11"/>
+    <hyperlink r:id="rId11" ref="D12"/>
+    <hyperlink r:id="rId12" ref="D13"/>
+    <hyperlink r:id="rId13" ref="D14"/>
+    <hyperlink r:id="rId14" ref="D15"/>
+    <hyperlink r:id="rId15" ref="D16"/>
+    <hyperlink r:id="rId16" ref="D17"/>
+    <hyperlink r:id="rId17" ref="D18"/>
+    <hyperlink r:id="rId18" ref="D19"/>
+    <hyperlink r:id="rId19" ref="D20"/>
+    <hyperlink r:id="rId20" ref="D21"/>
+    <hyperlink r:id="rId21" ref="D22"/>
+    <hyperlink r:id="rId22" ref="D23"/>
+    <hyperlink r:id="rId23" ref="D24"/>
+    <hyperlink r:id="rId24" ref="D25"/>
+    <hyperlink r:id="rId25" ref="D26"/>
+    <hyperlink r:id="rId26" ref="D27"/>
+    <hyperlink r:id="rId27" ref="D28"/>
+    <hyperlink r:id="rId28" ref="D29"/>
+    <hyperlink r:id="rId29" ref="D30"/>
+    <hyperlink r:id="rId30" ref="D31"/>
+    <hyperlink r:id="rId31" ref="D32"/>
+    <hyperlink r:id="rId32" ref="D33"/>
+    <hyperlink r:id="rId33" ref="D34"/>
+    <hyperlink r:id="rId34" ref="D35"/>
+    <hyperlink r:id="rId35" ref="D36"/>
+    <hyperlink r:id="rId36" ref="D37"/>
+    <hyperlink r:id="rId37" ref="D38"/>
+    <hyperlink r:id="rId38" ref="D39"/>
+    <hyperlink r:id="rId39" ref="D40"/>
+    <hyperlink r:id="rId40" ref="D41"/>
+    <hyperlink r:id="rId41" ref="D42"/>
+    <hyperlink r:id="rId42" ref="D43"/>
+    <hyperlink r:id="rId43" ref="B44"/>
+    <hyperlink r:id="rId44" ref="D44"/>
+    <hyperlink r:id="rId45" ref="D45"/>
+    <hyperlink r:id="rId46" ref="D46"/>
+    <hyperlink r:id="rId47" ref="D47"/>
+    <hyperlink r:id="rId48" ref="D48"/>
   </hyperlinks>
-  <drawing r:id="rId3"/>
+  <drawing r:id="rId49"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId51"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>